<commit_message>
Update reports and notebooks with latest data (2025)
- Refresh all China-PLP trade analysis notebooks
- Update country trade profiles with 2024-2025 data
- Regenerate Excel reports and charts
- Update partner/reporter reference files

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/China_2.1.1_top_export_partners_reverse.xlsx
+++ b/reports/China_2.1.1_top_export_partners_reverse.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7405" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7457" uniqueCount="198">
   <si>
     <t>refYear</t>
   </si>
@@ -965,7 +965,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J1850"/>
+  <dimension ref="A1:J1863"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -60165,6 +60165,422 @@
         <v>3237870084945.707</v>
       </c>
     </row>
+    <row r="1851" spans="1:10">
+      <c r="A1851" s="1">
+        <v>1855</v>
+      </c>
+      <c r="B1851">
+        <v>2025</v>
+      </c>
+      <c r="C1851" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1851" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1851">
+        <v>1</v>
+      </c>
+      <c r="F1851" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1851" t="s">
+        <v>197</v>
+      </c>
+      <c r="H1851">
+        <v>171247595342.999</v>
+      </c>
+      <c r="I1851">
+        <v>0.3220615711169312</v>
+      </c>
+      <c r="J1851">
+        <v>531723157001.007</v>
+      </c>
+    </row>
+    <row r="1852" spans="1:10">
+      <c r="A1852" s="1">
+        <v>1858</v>
+      </c>
+      <c r="B1852">
+        <v>2025</v>
+      </c>
+      <c r="C1852" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1852" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1852">
+        <v>2</v>
+      </c>
+      <c r="F1852" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1852" t="s">
+        <v>197</v>
+      </c>
+      <c r="H1852">
+        <v>133243185268</v>
+      </c>
+      <c r="I1852">
+        <v>0.2505875162923319</v>
+      </c>
+      <c r="J1852">
+        <v>531723157001.007</v>
+      </c>
+    </row>
+    <row r="1853" spans="1:10">
+      <c r="A1853" s="1">
+        <v>1854</v>
+      </c>
+      <c r="B1853">
+        <v>2025</v>
+      </c>
+      <c r="C1853" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1853" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1853">
+        <v>3</v>
+      </c>
+      <c r="F1853" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1853" t="s">
+        <v>197</v>
+      </c>
+      <c r="H1853">
+        <v>87535512266.754</v>
+      </c>
+      <c r="I1853">
+        <v>0.1646261049837786</v>
+      </c>
+      <c r="J1853">
+        <v>531723157001.007</v>
+      </c>
+    </row>
+    <row r="1854" spans="1:10">
+      <c r="A1854" s="1">
+        <v>1850</v>
+      </c>
+      <c r="B1854">
+        <v>2025</v>
+      </c>
+      <c r="C1854" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1854" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1854">
+        <v>4</v>
+      </c>
+      <c r="F1854" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1854" t="s">
+        <v>197</v>
+      </c>
+      <c r="H1854">
+        <v>75871729539</v>
+      </c>
+      <c r="I1854">
+        <v>0.1426902863642937</v>
+      </c>
+      <c r="J1854">
+        <v>531723157001.007</v>
+      </c>
+    </row>
+    <row r="1855" spans="1:10">
+      <c r="A1855" s="1">
+        <v>1861</v>
+      </c>
+      <c r="B1855">
+        <v>2025</v>
+      </c>
+      <c r="C1855" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1855" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1855">
+        <v>5</v>
+      </c>
+      <c r="F1855" t="s">
+        <v>38</v>
+      </c>
+      <c r="G1855" t="s">
+        <v>197</v>
+      </c>
+      <c r="H1855">
+        <v>24936545740.154</v>
+      </c>
+      <c r="I1855">
+        <v>0.04689761093122144</v>
+      </c>
+      <c r="J1855">
+        <v>531723157001.007</v>
+      </c>
+    </row>
+    <row r="1856" spans="1:10">
+      <c r="A1856" s="1">
+        <v>1859</v>
+      </c>
+      <c r="B1856">
+        <v>2025</v>
+      </c>
+      <c r="C1856" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1856" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1856">
+        <v>6</v>
+      </c>
+      <c r="F1856" t="s">
+        <v>52</v>
+      </c>
+      <c r="G1856" t="s">
+        <v>197</v>
+      </c>
+      <c r="H1856">
+        <v>13093508791.542</v>
+      </c>
+      <c r="I1856">
+        <v>0.02462467285681372</v>
+      </c>
+      <c r="J1856">
+        <v>531723157001.007</v>
+      </c>
+    </row>
+    <row r="1857" spans="1:10">
+      <c r="A1857" s="1">
+        <v>1852</v>
+      </c>
+      <c r="B1857">
+        <v>2025</v>
+      </c>
+      <c r="C1857" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1857" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1857">
+        <v>7</v>
+      </c>
+      <c r="F1857" t="s">
+        <v>62</v>
+      </c>
+      <c r="G1857" t="s">
+        <v>197</v>
+      </c>
+      <c r="H1857">
+        <v>12340526109.903</v>
+      </c>
+      <c r="I1857">
+        <v>0.02320855495462205</v>
+      </c>
+      <c r="J1857">
+        <v>531723157001.007</v>
+      </c>
+    </row>
+    <row r="1858" spans="1:10">
+      <c r="A1858" s="1">
+        <v>1860</v>
+      </c>
+      <c r="B1858">
+        <v>2025</v>
+      </c>
+      <c r="C1858" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1858" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1858">
+        <v>8</v>
+      </c>
+      <c r="F1858" t="s">
+        <v>77</v>
+      </c>
+      <c r="G1858" t="s">
+        <v>197</v>
+      </c>
+      <c r="H1858">
+        <v>6658050998.242</v>
+      </c>
+      <c r="I1858">
+        <v>0.01252164949105158</v>
+      </c>
+      <c r="J1858">
+        <v>531723157001.007</v>
+      </c>
+    </row>
+    <row r="1859" spans="1:10">
+      <c r="A1859" s="1">
+        <v>1857</v>
+      </c>
+      <c r="B1859">
+        <v>2025</v>
+      </c>
+      <c r="C1859" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1859" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1859">
+        <v>9</v>
+      </c>
+      <c r="F1859" t="s">
+        <v>109</v>
+      </c>
+      <c r="G1859" t="s">
+        <v>197</v>
+      </c>
+      <c r="H1859">
+        <v>2558404235</v>
+      </c>
+      <c r="I1859">
+        <v>0.004811534350750789</v>
+      </c>
+      <c r="J1859">
+        <v>531723157001.007</v>
+      </c>
+    </row>
+    <row r="1860" spans="1:10">
+      <c r="A1860" s="1">
+        <v>1851</v>
+      </c>
+      <c r="B1860">
+        <v>2025</v>
+      </c>
+      <c r="C1860" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1860" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1860">
+        <v>10</v>
+      </c>
+      <c r="F1860" t="s">
+        <v>150</v>
+      </c>
+      <c r="G1860" t="s">
+        <v>197</v>
+      </c>
+      <c r="H1860">
+        <v>1346916294.923</v>
+      </c>
+      <c r="I1860">
+        <v>0.002533115733608061</v>
+      </c>
+      <c r="J1860">
+        <v>531723157001.007</v>
+      </c>
+    </row>
+    <row r="1861" spans="1:10">
+      <c r="A1861" s="1">
+        <v>1853</v>
+      </c>
+      <c r="B1861">
+        <v>2025</v>
+      </c>
+      <c r="C1861" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1861" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1861">
+        <v>11</v>
+      </c>
+      <c r="F1861" t="s">
+        <v>131</v>
+      </c>
+      <c r="G1861" t="s">
+        <v>197</v>
+      </c>
+      <c r="H1861">
+        <v>1295445372.959</v>
+      </c>
+      <c r="I1861">
+        <v>0.002436315507237814</v>
+      </c>
+      <c r="J1861">
+        <v>531723157001.007</v>
+      </c>
+    </row>
+    <row r="1862" spans="1:10">
+      <c r="A1862" s="1">
+        <v>1856</v>
+      </c>
+      <c r="B1862">
+        <v>2025</v>
+      </c>
+      <c r="C1862" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1862" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1862">
+        <v>12</v>
+      </c>
+      <c r="F1862" t="s">
+        <v>126</v>
+      </c>
+      <c r="G1862" t="s">
+        <v>197</v>
+      </c>
+      <c r="H1862">
+        <v>1180369523.819</v>
+      </c>
+      <c r="I1862">
+        <v>0.002219894898835043</v>
+      </c>
+      <c r="J1862">
+        <v>531723157001.007</v>
+      </c>
+    </row>
+    <row r="1863" spans="1:10">
+      <c r="A1863" s="1">
+        <v>1849</v>
+      </c>
+      <c r="B1863">
+        <v>2025</v>
+      </c>
+      <c r="C1863" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1863" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1863">
+        <v>13</v>
+      </c>
+      <c r="F1863" t="s">
+        <v>189</v>
+      </c>
+      <c r="G1863" t="s">
+        <v>197</v>
+      </c>
+      <c r="H1863">
+        <v>415367517.712</v>
+      </c>
+      <c r="I1863">
+        <v>0.0007811725185239833</v>
+      </c>
+      <c r="J1863">
+        <v>531723157001.007</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>